<commit_message>
Replaced checkboxes with brackets and fixed colors
</commit_message>
<xml_diff>
--- a/data/habits.xlsx
+++ b/data/habits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,21 +468,203 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Drhello world ink Water</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Read Books</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>contact linkedin</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dont use instagram</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>i learned to build the app</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>doing good</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Lesson</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>learning</t>
         </is>
       </c>
-      <c r="D2" t="b">
+      <c r="D9" t="b">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed Perplexity API payload and QSS warnings
</commit_message>
<xml_diff>
--- a/data/habits.xlsx
+++ b/data/habits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,16 +598,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gratitude</t>
+          <t>Outreach</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>i learned to build the app</t>
+          <t>contack person</t>
         </is>
       </c>
       <c r="D7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>8</v>
@@ -629,7 +629,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>doing good</t>
+          <t>i learned to build the app</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -650,12 +650,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Gratitude</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>doing good</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -665,6 +665,80 @@
         <v>8</v>
       </c>
       <c r="F9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>helo</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>learning</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Read-Only History and Future Planning to Habit Tracker
</commit_message>
<xml_diff>
--- a/data/habits.xlsx
+++ b/data/habits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -515,17 +515,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Main Tasks</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>contact linkedin</t>
+          <t>hello world</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -541,7 +541,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -551,11 +551,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sdf</t>
+          <t>contact linkedin</t>
         </is>
       </c>
       <c r="D5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>8</v>
@@ -567,21 +567,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>dont use instagram</t>
+          <t>sdf</t>
         </is>
       </c>
       <c r="D6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>8</v>
@@ -593,7 +593,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>contack person</t>
+          <t>dont use instagram</t>
         </is>
       </c>
       <c r="D7" t="b">
@@ -619,21 +619,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gratitude</t>
+          <t>Outreach</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>i learned to build the app</t>
+          <t>contack person</t>
         </is>
       </c>
       <c r="D8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>8</v>
@@ -645,7 +645,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>doing good</t>
+          <t>i learned to build the app</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -671,7 +671,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>helo</t>
+          <t>doing good</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -697,7 +697,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -705,7 +705,11 @@
           <t>Gratitude</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>helo</t>
+        </is>
+      </c>
       <c r="D11" t="b">
         <v>1</v>
       </c>
@@ -719,26 +723,330 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>learning</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>2025-12-02</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Drhello world ink Water</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Read Books</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>contact linkedin</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dont use instagram</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>contack person</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>i learned to build the app</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>doing good</t>
+        </is>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>helo</t>
+        </is>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Lesson</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>learning</t>
         </is>
       </c>
-      <c r="D12" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>8</v>
-      </c>
-      <c r="F12" t="n">
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added multi-tab browser, footer command shell, and transition animations
</commit_message>
<xml_diff>
--- a/data/habits.xlsx
+++ b/data/habits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -781,17 +781,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Drhello world ink Water</t>
+          <t>Drink 5 bottles of water</t>
         </is>
       </c>
       <c r="D14" t="b">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -807,17 +807,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Read Books</t>
+          <t>Take bath</t>
         </is>
       </c>
       <c r="D15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -828,22 +828,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Main Tasks</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>contact linkedin</t>
+          <t>Eat pg food only</t>
         </is>
       </c>
       <c r="D16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -854,22 +854,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Main Tasks</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sdf</t>
+          <t>No porns</t>
         </is>
       </c>
       <c r="D17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -880,22 +880,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>dont use instagram</t>
+          <t>PG RENT PAID 7500</t>
         </is>
       </c>
       <c r="D18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -906,22 +906,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>contack person</t>
+          <t>Complete the daily task manager app</t>
         </is>
       </c>
       <c r="D19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -932,22 +932,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gratitude</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>i learned to build the app</t>
+          <t>Study ROS2 for 1 hour</t>
         </is>
       </c>
       <c r="D20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -958,22 +958,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Gratitude</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>doing good</t>
+          <t>Study DS from 9.30 pm to onwards from codingninja</t>
         </is>
       </c>
       <c r="D21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -984,22 +984,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Gratitude</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>helo</t>
+          <t>Learn ML pipelines and note down in notebook</t>
         </is>
       </c>
       <c r="D22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -1010,18 +1010,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gratitude</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Apply for job - 5</t>
+        </is>
+      </c>
       <c r="D23" t="b">
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -1032,22 +1036,482 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Use notebook while learning</t>
+        </is>
+      </c>
+      <c r="D24" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>For having good life</t>
+        </is>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>For getting job</t>
+        </is>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To learn saving </t>
+        </is>
+      </c>
+      <c r="D27" t="b">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Lesson</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>learning</t>
-        </is>
-      </c>
-      <c r="D24" t="b">
-        <v>1</v>
-      </c>
-      <c r="E24" t="n">
-        <v>8</v>
-      </c>
-      <c r="F24" t="n">
-        <v>10</v>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fake it till you make it; </t>
+        </is>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Wake up 5AM</t>
+        </is>
+      </c>
+      <c r="D29" t="b">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Drink 5 bottles of water</t>
+        </is>
+      </c>
+      <c r="D30" t="b">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pushup and body exercise</t>
+        </is>
+      </c>
+      <c r="D31" t="b">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>No porns</t>
+        </is>
+      </c>
+      <c r="D32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PG food only</t>
+        </is>
+      </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Protocols</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>NO sleeping before 12 night and no sleeping in daytime</t>
+        </is>
+      </c>
+      <c r="D34" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ROS2 for 1 hour</t>
+        </is>
+      </c>
+      <c r="D35" t="b">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DS for 3 hours</t>
+        </is>
+      </c>
+      <c r="D36" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Main Tasks</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Apply for job - 10</t>
+        </is>
+      </c>
+      <c r="D38" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Don't message her</t>
+        </is>
+      </c>
+      <c r="D39" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For learning and upskill </t>
+        </is>
+      </c>
+      <c r="D41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>For plan to Germany</t>
+        </is>
+      </c>
+      <c r="D42" t="b">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chatbot Offline Mode: Input disable and friendly errors
</commit_message>
<xml_diff>
--- a/data/habits.xlsx
+++ b/data/habits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="D20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>5</v>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fake it till you make it; </t>
+          <t>Fake it till you make it; have to improve a lot as I am ignoring all things, I need to control thoughts and actions.</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -1322,16 +1322,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Main Tasks</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ROS2 for 1 hour</t>
+          <t>Take a bath</t>
         </is>
       </c>
       <c r="D35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>5</v>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DS for 3 hours</t>
+          <t>ROS2 for 1 hour</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -1377,7 +1377,11 @@
           <t>Main Tasks</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DS for 3 hours</t>
+        </is>
+      </c>
       <c r="D37" t="b">
         <v>0</v>
       </c>
@@ -1396,12 +1400,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Apply for job - 10</t>
+          <t>Make the laptop storage clean</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -1422,12 +1426,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Don't message her</t>
+          <t>ML pipeline learning</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -1451,7 +1455,11 @@
           <t>Outreach</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Apply for job - 10</t>
+        </is>
+      </c>
       <c r="D40" t="b">
         <v>0</v>
       </c>
@@ -1470,16 +1478,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Gratitude</t>
+          <t>Outreach</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">For learning and upskill </t>
+          <t>Don't message her</t>
         </is>
       </c>
       <c r="D41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E41" t="n">
         <v>5</v>
@@ -1496,21 +1504,73 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Go for walk in the evening</t>
+        </is>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>Gratitude</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For learning and upskill </t>
+        </is>
+      </c>
+      <c r="D43" t="b">
+        <v>1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Gratitude</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
         <is>
           <t>For plan to Germany</t>
         </is>
       </c>
-      <c r="D42" t="b">
-        <v>1</v>
-      </c>
-      <c r="E42" t="n">
-        <v>5</v>
-      </c>
-      <c r="F42" t="n">
+      <c r="D44" t="b">
+        <v>1</v>
+      </c>
+      <c r="E44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feature: Real-time Data Sync between TaskPage and DashboardPage using Router signal
</commit_message>
<xml_diff>
--- a/data/habits.xlsx
+++ b/data/habits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2102,12 +2102,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Main Tasks</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Apply for job - 10</t>
+          <t>AI interview practice</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -2133,16 +2133,42 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
+          <t>Apply for job - 10</t>
+        </is>
+      </c>
+      <c r="D66" t="b">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
           <t>Go for walk in the evening</t>
         </is>
       </c>
-      <c r="D66" t="b">
-        <v>0</v>
-      </c>
-      <c r="E66" t="n">
-        <v>5</v>
-      </c>
-      <c r="F66" t="n">
+      <c r="D67" t="b">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>5</v>
+      </c>
+      <c r="F67" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>